<commit_message>
Calculo de Potencia Inversor, add Zona 5 (Calefaccion)
</commit_message>
<xml_diff>
--- a/data/BBDD_Equipos.xlsx
+++ b/data/BBDD_Equipos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29303"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardo/Documents/Proyectos/Solar/Sprint7_PerfilBase_v1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardo/Documents/Proyectos/Solar/KVA2/KVA-Beta/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{38690B94-E4CA-444F-819A-167BEFDF213C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50DE07EF-6DFF-47C2-B3ED-D7392F5CA5CD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5967A59-DF23-A340-975A-32910521EEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50980" yWindow="660" windowWidth="30240" windowHeight="17300" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50980" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paneles" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="158">
   <si>
     <t>Marca</t>
   </si>
@@ -510,6 +510,9 @@
   </si>
   <si>
     <t>BlueSolar MPPT 150/70-TR</t>
+  </si>
+  <si>
+    <t>Inventado</t>
   </si>
 </sst>
 </file>
@@ -517,11 +520,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="[$$-340A]#,##0"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="[$$-340A]#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -807,7 +810,7 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -875,15 +878,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -891,17 +894,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -1210,19 +1213,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EB4E075-28A8-4E64-A219-D8FBC6D6FB1F}">
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" customWidth="1"/>
-    <col min="5" max="5" width="25.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="18.42578125" customWidth="1"/>
-    <col min="11" max="11" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.5" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="33.6" customHeight="1" thickBot="1">
+    <row r="1" spans="1:12" ht="33.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14"/>
       <c r="B1" s="15" t="s">
         <v>0</v>
@@ -1256,7 +1259,7 @@
       </c>
       <c r="L1" s="6"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -1291,7 +1294,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -1326,7 +1329,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -1361,7 +1364,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -1396,7 +1399,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -1466,7 +1469,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -1501,7 +1504,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -1536,7 +1539,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -1571,7 +1574,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -1606,7 +1609,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -1641,7 +1644,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -1676,7 +1679,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -1711,7 +1714,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -1746,7 +1749,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>15</v>
       </c>
@@ -1781,7 +1784,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>16</v>
       </c>
@@ -1816,7 +1819,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -1851,7 +1854,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>18</v>
       </c>
@@ -1886,7 +1889,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -1921,7 +1924,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.95" thickBot="1">
+    <row r="21" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>20</v>
       </c>
@@ -1956,7 +1959,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1967,7 +1970,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="1"/>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1978,7 +1981,7 @@
       <c r="I25" s="5"/>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -1989,7 +1992,7 @@
       <c r="I26" s="5"/>
       <c r="J26" s="1"/>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1999,7 +2002,7 @@
       <c r="H27" s="3"/>
       <c r="I27" s="5"/>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28" s="4"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -2038,21 +2041,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F61D9440-0025-46A2-B042-DF977E776D37}">
-  <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.33203125" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" customWidth="1"/>
-    <col min="6" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="6" max="7" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="44.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="34.5" customHeight="1">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2081,7 +2084,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2113,7 +2116,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2145,7 +2148,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2177,7 +2180,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2209,7 +2212,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2241,7 +2244,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2273,7 +2276,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2305,7 +2308,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2337,7 +2340,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2369,7 +2372,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2401,7 +2404,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2433,7 +2436,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2465,7 +2468,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2497,7 +2500,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2529,7 +2532,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2561,7 +2564,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2619,7 +2622,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2645,7 +2648,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2668,6 +2671,32 @@
         <v>87</v>
       </c>
       <c r="H20" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D21">
+        <v>25000</v>
+      </c>
+      <c r="E21">
+        <v>48</v>
+      </c>
+      <c r="F21">
+        <v>3419000</v>
+      </c>
+      <c r="G21" t="s">
+        <v>87</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2687,26 +2716,27 @@
     <hyperlink ref="H16" r:id="rId12" xr:uid="{C70BFDA3-BECF-4640-980B-54BA68137494}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CD261A6-7F5F-473D-99A1-B9C6417D22AC}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="68.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="68.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="25"/>
       <c r="B1" s="26" t="s">
         <v>0</v>
@@ -2733,7 +2763,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="34">
         <v>1</v>
       </c>
@@ -2762,7 +2792,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="39">
         <v>2</v>
       </c>
@@ -2791,7 +2821,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="39">
         <v>3</v>
       </c>
@@ -2820,7 +2850,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="34">
         <v>4</v>
       </c>
@@ -2849,7 +2879,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="39">
         <v>5</v>
       </c>
@@ -2878,7 +2908,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="39">
         <v>6</v>
       </c>
@@ -2918,19 +2948,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA6FBE73-61D9-450C-8B32-B1D20EAB2AC0}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.5" customWidth="1"/>
+    <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5" style="30" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="48.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.1">
+    <row r="1" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="19"/>
       <c r="B1" s="15" t="s">
         <v>0</v>
@@ -2957,7 +2987,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -2986,7 +3016,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -3015,7 +3045,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -3044,7 +3074,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -3073,7 +3103,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -3102,7 +3132,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -3131,7 +3161,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -3160,7 +3190,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -3189,7 +3219,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.95" thickBot="1">
+    <row r="10" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>9</v>
       </c>
@@ -3218,50 +3248,50 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D13" s="23"/>
       <c r="E13" s="29"/>
       <c r="F13" s="30"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E14" s="29"/>
       <c r="F14" s="30"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E15" s="29"/>
       <c r="F15" s="30"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E16" s="29"/>
       <c r="F16" s="30"/>
     </row>
-    <row r="17" spans="5:6">
+    <row r="17" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E17" s="29"/>
       <c r="F17" s="30"/>
     </row>
-    <row r="18" spans="5:6">
+    <row r="18" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E18" s="29"/>
       <c r="F18" s="30"/>
     </row>
-    <row r="19" spans="5:6">
+    <row r="19" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E19" s="29"/>
       <c r="F19" s="30"/>
     </row>
-    <row r="20" spans="5:6">
+    <row r="20" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E20" s="29"/>
       <c r="F20" s="30"/>
     </row>
-    <row r="21" spans="5:6">
+    <row r="21" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E21" s="29"/>
       <c r="F21" s="30"/>
     </row>
-    <row r="22" spans="5:6">
+    <row r="22" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E22" s="29"/>
     </row>
-    <row r="23" spans="5:6">
+    <row r="23" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E23" s="29"/>
     </row>
-    <row r="24" spans="5:6">
+    <row r="24" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E24" s="29"/>
     </row>
   </sheetData>
@@ -3270,6 +3300,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Participa xmlns="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53">true</Participa>
+    <TaxCatchAll xmlns="e8d2ff9b-5f5c-45a4-9648-827360dcfaf3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AA99E0A26634CB42BEA9C6EBCCC3F3D9" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="418a5ed0b0c744fdec2080f7385043f1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53" xmlns:ns3="e8d2ff9b-5f5c-45a4-9648-827360dcfaf3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1a7dadd62680cb5ee6dd0a3d1712cdf6" ns2:_="" ns3:_="">
     <xsd:import namespace="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53"/>
@@ -3488,35 +3539,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Participa xmlns="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53">true</Participa>
-    <TaxCatchAll xmlns="e8d2ff9b-5f5c-45a4-9648-827360dcfaf3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F4EFD3C-C58B-4B45-B6F9-7FE4F5A52AE1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{836E8950-B34B-43F5-AF7E-94CCC98D4EC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53"/>
+    <ds:schemaRef ds:uri="e8d2ff9b-5f5c-45a4-9648-827360dcfaf3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FEB314F-088A-4857-BE2A-E6026359DCDD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FEB314F-088A-4857-BE2A-E6026359DCDD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{836E8950-B34B-43F5-AF7E-94CCC98D4EC7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F4EFD3C-C58B-4B45-B6F9-7FE4F5A52AE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2e14f83a-67ec-4bc9-9da1-ece74f6f9d53"/>
+    <ds:schemaRef ds:uri="e8d2ff9b-5f5c-45a4-9648-827360dcfaf3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>